<commit_message>
ssh-git-client -- documentation, and fix minor askpass bug
</commit_message>
<xml_diff>
--- a/docs/SSH-folder-documentation.xlsx
+++ b/docs/SSH-folder-documentation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jan/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jan/Documents/Projects/Pragma-git/pragma-git/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9966F260-B685-514C-896F-00BECDBFF406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B00A067-CEEB-544D-B4D0-EF01A828C1AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2900" yWindow="7380" windowWidth="29140" windowHeight="25700" xr2:uid="{C613FC87-67E9-B343-A3B4-DE82EF5D14EE}"/>
+    <workbookView xWindow="2900" yWindow="880" windowWidth="29140" windowHeight="25700" xr2:uid="{C613FC87-67E9-B343-A3B4-DE82EF5D14EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="58">
   <si>
     <t>System</t>
   </si>
@@ -74,9 +74,6 @@
     <t>/tmp/pragma-git-ssh-folders</t>
   </si>
   <si>
-    <t>delayed-start-pragma-merge</t>
-  </si>
-  <si>
     <t>ssh-close-pragma-merge-ssh</t>
   </si>
   <si>
@@ -86,9 +83,6 @@
     <t>ssh-get</t>
   </si>
   <si>
-    <t>ssh-get-merge-files</t>
-  </si>
-  <si>
     <t>ssh-git-client</t>
   </si>
   <si>
@@ -105,9 +99,6 @@
   </si>
   <si>
     <t>sourced in most of above scripts</t>
-  </si>
-  <si>
-    <t>lib/</t>
   </si>
   <si>
     <t>ssh-functions</t>
@@ -275,12 +266,6 @@
     </r>
   </si>
   <si>
-    <t>Started from ssh-git-client -&gt; delayed-start-pragma-merge -&gt; ssh-get-merge-files</t>
-  </si>
-  <si>
-    <t>ssh-git-client -&gt; delayed-start-pragma-merge -&gt; ssh-get-merge-files</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Runs this if git command contains </t>
     </r>
@@ -296,16 +281,175 @@
   </si>
   <si>
     <r>
-      <t>Started by "</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
+      <t xml:space="preserve">ssh-get-merge-files  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(ends by calling </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <rFont val="Courier New"/>
         <family val="1"/>
       </rPr>
-      <t>delayed-start-pragma-merge</t>
+      <t>pragma-merge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>=&gt;</t>
+    </r>
+  </si>
+  <si>
+    <t>pragma-merge (called by ssh-get-merge-files)</t>
+  </si>
+  <si>
+    <t>WINDOWS -- Clicking (diff) link  in list of modified files, the following should happen for an ssh-folder:</t>
+  </si>
+  <si>
+    <t>WINDOWS</t>
+  </si>
+  <si>
+    <t>ssh-close-pragma-merge-ssh (called from app.js, when closing Pragma-merge GUI)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">Created:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>C:\Users\axels\AppData\Local\Temp\pragma-git-ssh-folders\tmp\git-blob*</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">Created:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>C:\Users\axels\AppData\Local\Temp\pragma-git-ssh-folders\*</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In WSL console:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>tail -f /mnt/c/Users/axels/.Pragma-git/.tmp/ssh-log.log</t>
+    </r>
+  </si>
+  <si>
+    <t>TODO : Which EXIT CODE should be returned?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To log opening and closing Pragma-git from list of modified files : </t>
+  </si>
+  <si>
+    <t>called by pragma-merge.js if [Save] button pressed</t>
+  </si>
+  <si>
+    <t>Copied file  from server to here</t>
+  </si>
+  <si>
+    <t>Copied git-blobs from server to here</t>
+  </si>
+  <si>
+    <t>Put file relative TEMP_FILE_LOCATION/ into repo</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In WSL console:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="1"/>
+      </rPr>
+      <t>tail -f /mnt/c/Users/axels/.Pragma-git/.tmp/mergelog.log</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ssh-log from ssh-git-client </t>
+  </si>
+  <si>
+    <t>LOGS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ssh-git-client -&gt; ssh-get-merge-files </t>
+  </si>
+  <si>
+    <t>Started from ssh-git-client, when poll shows that git has called the pragma-merge command</t>
+  </si>
+  <si>
+    <t>in pragma-git folder</t>
+  </si>
+  <si>
+    <t>./ssh-folders/lib/</t>
+  </si>
+  <si>
+    <t>bash</t>
+  </si>
+  <si>
+    <t>MacOS, Linux runs in local host so it is uncomplicated -- Windows bash commands runs in WSL</t>
+  </si>
+  <si>
+    <r>
+      <t>Assuming remote is called</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Linux</t>
     </r>
     <r>
       <rPr>
@@ -315,192 +459,37 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>" (which runs ssh-get-merge-files after 2 seconds)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">ssh-get-merge-files  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
+      <t xml:space="preserve">, and local is called </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">(ends by calling </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Courier New"/>
-        <family val="1"/>
-      </rPr>
-      <t>pragma-merge</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="9"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>bash</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>=&gt;</t>
-    </r>
-  </si>
-  <si>
-    <t>pragma-merge (called by ssh-get-merge-files)</t>
-  </si>
-  <si>
-    <t>WINDOWS -- Clicking (diff) link  in list of modified files, the following should happen for an ssh-folder:</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Assuming remote is called</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Linux</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, and local is called </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>WSL</t>
-    </r>
-  </si>
-  <si>
-    <t>WINDOWS</t>
-  </si>
-  <si>
-    <t>ssh-close-pragma-merge-ssh (called from app.js, when closing Pragma-merge GUI)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve">Created:  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="1"/>
-      </rPr>
-      <t>C:\Users\axels\AppData\Local\Temp\pragma-git-ssh-folders\tmp\git-blob*</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve">Created:  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="1"/>
-      </rPr>
-      <t>C:\Users\axels\AppData\Local\Temp\pragma-git-ssh-folders\*</t>
-    </r>
-  </si>
-  <si>
-    <t>WINDOWS behavior    (MacOS, Linux runs in local host so it is uncomplicated -- Windows bash commands runs in WSL)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">In WSL console:  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="1"/>
-      </rPr>
-      <t>tail -f /mnt/c/Users/axels/.Pragma-git/.tmp/ssh-log.log</t>
-    </r>
-  </si>
-  <si>
-    <t>TODO : Which EXIT CODE should be returned?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">To log opening and closing Pragma-git from list of modified files : </t>
-  </si>
-  <si>
-    <t>called by pragma-merge.js if [Save] button pressed</t>
-  </si>
-  <si>
-    <t>Copied file  from server to here</t>
-  </si>
-  <si>
-    <t>Copied git-blobs from server to here</t>
-  </si>
-  <si>
-    <t>Put file relative TEMP_FILE_LOCATION/ into repo</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">In WSL console:  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Courier New"/>
-        <family val="1"/>
-      </rPr>
-      <t>tail -f /mnt/c/Users/axels/.Pragma-git/.tmp/mergelog.log</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">ssh-log from ssh-git-client </t>
-  </si>
-  <si>
-    <t>LOGS</t>
+      <t>"</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -524,13 +513,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
@@ -632,6 +614,12 @@
       <sz val="12"/>
       <name val="Courier New"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="9"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="3">
@@ -728,53 +716,49 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="4"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="6"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="4"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -813,7 +797,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CE091524-643B-4A4A-9433-2397E6D759EA}" name="Table2" displayName="Table2" ref="B3:D7" totalsRowShown="0" headerRowCellStyle="Accent1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CE091524-643B-4A4A-9433-2397E6D759EA}" name="Table2" displayName="Table2" ref="B3:D7" totalsRowShown="0">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{720B33F4-6726-864D-B680-EDFAC77EB12B}" name="System" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{26584A06-CB5E-EC44-82F5-AF833181D3C3}" name="Normal Temp Folder -- TMP in bash scripts" dataDxfId="0"/>
@@ -1140,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B047B3B7-057A-C840-91B5-E68C7414CEFE}">
-  <dimension ref="A3:D61"/>
+  <dimension ref="A3:D59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="13.1640625" customWidth="1"/>
@@ -1153,7 +1137,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>1</v>
@@ -1161,20 +1145,20 @@
     </row>
     <row r="4" spans="2:4" ht="17">
       <c r="B4" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="17">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="19"/>
     </row>
     <row r="6" spans="2:4" ht="17">
       <c r="B6" s="9" t="s">
@@ -1203,22 +1187,22 @@
         <v>0</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="17">
-      <c r="B11" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
+      <c r="B11" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="28"/>
+      <c r="D11" s="29"/>
     </row>
     <row r="12" spans="2:4" ht="17">
-      <c r="B12" s="27" t="s">
-        <v>44</v>
+      <c r="B12" s="23" t="s">
+        <v>37</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>9</v>
@@ -1226,7 +1210,7 @@
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="2:4" ht="17">
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="16" t="s">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
@@ -1255,26 +1239,28 @@
     <row r="19" spans="1:4">
       <c r="B19" s="10"/>
       <c r="C19" s="4" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="D19" s="5"/>
     </row>
     <row r="20" spans="1:4" ht="17">
       <c r="B20" s="11"/>
       <c r="C20" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D20" s="2"/>
+        <v>19</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="21" spans="1:4" ht="17">
-      <c r="B21" s="19" t="s">
-        <v>3</v>
+      <c r="B21" s="16" t="s">
+        <v>55</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="17">
@@ -1284,56 +1270,56 @@
     </row>
     <row r="23" spans="1:4" ht="17">
       <c r="B23" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="17">
+      <c r="B24" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="17">
-      <c r="B24" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>28</v>
-      </c>
     </row>
     <row r="25" spans="1:4" ht="17">
-      <c r="A25" s="31"/>
-      <c r="B25" s="19" t="s">
-        <v>3</v>
+      <c r="A25" s="26"/>
+      <c r="B25" s="16" t="s">
+        <v>55</v>
       </c>
       <c r="C25" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="17">
+      <c r="B26" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="1:4" ht="17">
+      <c r="B27" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="17">
-      <c r="B26" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D26" s="2"/>
-    </row>
-    <row r="27" spans="1:4" ht="17">
-      <c r="B27" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>20</v>
-      </c>
       <c r="D27" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="17">
@@ -1342,219 +1328,197 @@
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" ht="17">
-      <c r="A29" s="25"/>
-      <c r="B29" s="19" t="s">
-        <v>3</v>
+      <c r="A29" s="26"/>
+      <c r="B29" s="16" t="s">
+        <v>55</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="2"/>
+      <c r="D29" s="25" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="30" spans="1:4" ht="17">
-      <c r="B30" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C30" s="13" t="s">
+      <c r="B30" s="16"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:4" ht="17">
+      <c r="B31" s="16"/>
+      <c r="C31" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" ht="17">
+      <c r="B32" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="17">
+      <c r="B33" s="11"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="1:4" ht="17">
+      <c r="B34" s="11"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="2"/>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="B36" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C36" s="4"/>
+      <c r="D36" s="5"/>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="B37" s="20"/>
+      <c r="C37" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="1:4" ht="17">
+      <c r="B38" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C38" s="13"/>
+      <c r="D38" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="17">
+      <c r="A39" s="26"/>
+      <c r="B39" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="17">
+      <c r="A40" s="26"/>
+      <c r="B40" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:4" ht="17">
+      <c r="A41" s="26"/>
+      <c r="B41" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C41" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:4" ht="17">
+      <c r="B42" s="20"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="1:4" ht="17">
+      <c r="B43" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C43" s="21"/>
+      <c r="D43" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="17">
+      <c r="B44" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="17">
+      <c r="B45" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="17">
+      <c r="B46" s="11"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="2"/>
+    </row>
+    <row r="47" spans="1:4" ht="17">
+      <c r="B47" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C47" s="21"/>
+      <c r="D47" s="2"/>
+    </row>
+    <row r="48" spans="1:4" ht="17">
+      <c r="B48" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D30" s="2"/>
-    </row>
-    <row r="31" spans="1:4" ht="17">
-      <c r="A31" s="31"/>
-      <c r="B31" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="30" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="17">
-      <c r="B32" s="19"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" spans="1:4" ht="17">
-      <c r="B33" s="19"/>
-      <c r="C33" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="1:4" ht="17">
-      <c r="B34" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="17">
-      <c r="B35" s="11"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="1:4" ht="17">
-      <c r="B36" s="11"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="2"/>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="B38" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="5"/>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="B39" s="23"/>
-      <c r="C39" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="D39" s="2"/>
-    </row>
-    <row r="40" spans="1:4" ht="17">
-      <c r="B40" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="C40" s="13"/>
-      <c r="D40" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="17">
-      <c r="A41" s="31"/>
-      <c r="B41" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="C41" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="17">
-      <c r="A42" s="31"/>
-      <c r="B42" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="C42" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="D42" s="2"/>
-    </row>
-    <row r="43" spans="1:4" ht="17">
-      <c r="A43" s="31"/>
-      <c r="B43" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="C43" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="D43" s="2"/>
-    </row>
-    <row r="44" spans="1:4" ht="17">
-      <c r="B44" s="23"/>
-      <c r="C44" s="24"/>
-      <c r="D44" s="2"/>
-    </row>
-    <row r="45" spans="1:4" ht="17">
-      <c r="B45" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="C45" s="24"/>
-      <c r="D45" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="17">
-      <c r="B46" s="29" t="s">
+      <c r="C48" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="17">
-      <c r="B47" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C47" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="17">
-      <c r="B48" s="11"/>
-      <c r="C48" s="24"/>
       <c r="D48" s="2"/>
     </row>
     <row r="49" spans="2:4" ht="17">
-      <c r="B49" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C49" s="24"/>
+      <c r="B49" s="11"/>
+      <c r="C49" s="21"/>
       <c r="D49" s="2"/>
     </row>
     <row r="50" spans="2:4" ht="17">
       <c r="B50" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C50" s="24" t="s">
-        <v>52</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="C50" s="21"/>
       <c r="D50" s="2"/>
     </row>
     <row r="51" spans="2:4" ht="17">
       <c r="B51" s="11"/>
-      <c r="C51" s="24"/>
+      <c r="C51" s="21"/>
       <c r="D51" s="2"/>
     </row>
-    <row r="52" spans="2:4" ht="17">
-      <c r="B52" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C52" s="24"/>
-      <c r="D52" s="2"/>
-    </row>
-    <row r="53" spans="2:4" ht="17">
-      <c r="B53" s="11"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="2"/>
-    </row>
-    <row r="57" spans="2:4">
-      <c r="B57" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C57" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="58" spans="2:4" ht="17">
+    <row r="55" spans="2:4">
+      <c r="B55" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C55" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" ht="17">
+      <c r="C56" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4">
       <c r="C58" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="60" spans="2:4">
-      <c r="C60" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="61" spans="2:4" ht="17">
-      <c r="C61" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" ht="17">
+      <c r="C59" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>